<commit_message>
Se culmino la primera parte de la limpieza de productos
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\La Fuente Estadistic\Desktop\INLASER-LA FUENTE\General_Analytics\Administracion\Administracion_Fuente\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\La Fuente Estadistic\Desktop\INLASER-LA FUENTE\General_Analytics\Contabilidad_Fuente\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA15F258-68A0-4228-99DF-51F4137E630F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A28C50-1DF2-4F47-8A73-C27939C6A19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$D$1312</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$D$1405</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5248" uniqueCount="2335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5582" uniqueCount="2463">
   <si>
     <t>PRODUCTO</t>
   </si>
@@ -7028,6 +7028,390 @@
   </si>
   <si>
     <t>AYUDA ELECTRÓNICA (BAJA VISIÓN)</t>
+  </si>
+  <si>
+    <t>ODONTOLOGIA</t>
+  </si>
+  <si>
+    <t>EXAMEN CLÍNICO</t>
+  </si>
+  <si>
+    <t>RAD. INTRAORAL</t>
+  </si>
+  <si>
+    <t>PROCEDIMIENTO</t>
+  </si>
+  <si>
+    <t>RESINA SIMPLE</t>
+  </si>
+  <si>
+    <t>RESINA COMPUESTA</t>
+  </si>
+  <si>
+    <t>RESINA COMPLEJA</t>
+  </si>
+  <si>
+    <t>FERULIZ. X PIEZA DENTAL</t>
+  </si>
+  <si>
+    <t>OPERATORIA</t>
+  </si>
+  <si>
+    <t>ENDODONCIA UNIRRADICULAR</t>
+  </si>
+  <si>
+    <t>ENDODONCIA MULTIRADICULAR</t>
+  </si>
+  <si>
+    <t>APICECTOMIA</t>
+  </si>
+  <si>
+    <t>ENDODONCIAS</t>
+  </si>
+  <si>
+    <t>PULPECTOMIA (INC. CORONA)</t>
+  </si>
+  <si>
+    <t>PULPOTOMIA CON RESTAURACION</t>
+  </si>
+  <si>
+    <t>PULPOTOMIA (INCLUYE CORONA)</t>
+  </si>
+  <si>
+    <t>MANTENEDOR DE ESPACIOS</t>
+  </si>
+  <si>
+    <t>INACT. CARIES DENTAL</t>
+  </si>
+  <si>
+    <t>SEDACION (ORAL)</t>
+  </si>
+  <si>
+    <t>ODONTOPEDIATRIA</t>
+  </si>
+  <si>
+    <t>EXODONCIA SIMPLE + PRF</t>
+  </si>
+  <si>
+    <t>EXODONCIA C/SUTURA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXODONCIA COMPLEJA 3ER MOLAR </t>
+  </si>
+  <si>
+    <t>EXODON. COMP. 3ER MOLAR ERUP.</t>
+  </si>
+  <si>
+    <t>CIRUGIA FRENILLO LINGUAL</t>
+  </si>
+  <si>
+    <t>CIRUGIA FRENILLO LABIAL</t>
+  </si>
+  <si>
+    <t>GINGIVOPLAST. (ELECTRO CIRUGIA)</t>
+  </si>
+  <si>
+    <t>OPERCULECTOMIA</t>
+  </si>
+  <si>
+    <t>CIRUGIAS</t>
+  </si>
+  <si>
+    <t>PROFILAXIS TOTAL ADULTO</t>
+  </si>
+  <si>
+    <t>PROFILAXIS PARCIAL ADULTO</t>
+  </si>
+  <si>
+    <t>PROFILAXIS NIÑOS (0-8 AÑOS)</t>
+  </si>
+  <si>
+    <t>PROFILAXIS NIÑOS (9-14 AÑOS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLUORIZACION X SESION </t>
+  </si>
+  <si>
+    <t>FLUORIZACION CON FLUOR BARNIZ</t>
+  </si>
+  <si>
+    <t>FLUORIZACION (CLIMPRO - VOCO )</t>
+  </si>
+  <si>
+    <t>BLANQ. DENTAL C/CUBETA INDIV+(1KIT)</t>
+  </si>
+  <si>
+    <t>KIT ADICIONAL DE 4 JERINGAS</t>
+  </si>
+  <si>
+    <t>BLANQUEAMIENTO SOLO GEL (EXTRA)</t>
+  </si>
+  <si>
+    <t>BLANQUEAMIENTO DENTAL A LASER</t>
+  </si>
+  <si>
+    <t>RASP. RADICULAR A CIELO ABIERTO X PIEZA</t>
+  </si>
+  <si>
+    <t>CORONA METAL PORCELANA</t>
+  </si>
+  <si>
+    <t>CORONA EN IVOCRON</t>
+  </si>
+  <si>
+    <t>CORONA LIBRE DE METAL EMAX</t>
+  </si>
+  <si>
+    <t>CORONA EN ZIRCONIO</t>
+  </si>
+  <si>
+    <t>CORONA METAL COMPLETA</t>
+  </si>
+  <si>
+    <t>CORONA EN PMMA</t>
+  </si>
+  <si>
+    <t>CORONA FENESTRADA</t>
+  </si>
+  <si>
+    <t>PERNO FIBRA DE VIDRIO/COLADO</t>
+  </si>
+  <si>
+    <t>INCRUSTACION EN IVOCRON</t>
+  </si>
+  <si>
+    <t>INCRUSTACION EN CEROMERO</t>
+  </si>
+  <si>
+    <t>INCRUSTACION EN EMAX</t>
+  </si>
+  <si>
+    <t>INCRUSTACION EN ZIRCONIO</t>
+  </si>
+  <si>
+    <t>CEMENTACION COR. C/CEMENTO FUJI/MERON</t>
+  </si>
+  <si>
+    <t>CEM.COR.LIB.MET.(CEM DUAL/RELIX/NEXUS RMGI)</t>
+  </si>
+  <si>
+    <t>RESINA SIMPLE EN PROTESIS FIJA</t>
+  </si>
+  <si>
+    <t>RESINA COMPUESTA PROTESIS FIJA</t>
+  </si>
+  <si>
+    <t>PROTECTOR OCLUSAL (FERULA OCLUSAL)</t>
+  </si>
+  <si>
+    <t>PROTESIS FIJA</t>
+  </si>
+  <si>
+    <t>PPR SUPERIOR MEJORADA</t>
+  </si>
+  <si>
+    <t>PPR INFERIOR MEJORADA</t>
+  </si>
+  <si>
+    <t>PPR CON ATACHE SUPERIOR MEJORADA</t>
+  </si>
+  <si>
+    <t>PPR CON ATACHE INFERIOR MEJORADA</t>
+  </si>
+  <si>
+    <t>PPR NORMAL SUPERIOR</t>
+  </si>
+  <si>
+    <t>PPR NORMAL INFERIOR</t>
+  </si>
+  <si>
+    <t>REBASE DE PPR SUPERIOR</t>
+  </si>
+  <si>
+    <t>REBASE DE PPR INFERIOR</t>
+  </si>
+  <si>
+    <t>PROTESIS PARCIAL REMOVIBLE</t>
+  </si>
+  <si>
+    <t>PPT MEJORADA SUPERIOR</t>
+  </si>
+  <si>
+    <t>PPT MEJORADA INFERIOR</t>
+  </si>
+  <si>
+    <t>PPT NORMAL SUPERIOR</t>
+  </si>
+  <si>
+    <t>PPT NORMAL INFERIOR</t>
+  </si>
+  <si>
+    <t>REBASE DE PROTESIS TOTAL SUPERIOR</t>
+  </si>
+  <si>
+    <t>REBASE DE PROTESIS TOTAL INFERIOR</t>
+  </si>
+  <si>
+    <t>PROTESIS TOTALES</t>
+  </si>
+  <si>
+    <t>IMPLANTE  CON REHABILITACION CON CORONA</t>
+  </si>
+  <si>
+    <t>IMPLANTE INMEDIATO</t>
+  </si>
+  <si>
+    <t>INJERTO DE TEJIDO CONECTIVO</t>
+  </si>
+  <si>
+    <t>INJERTO DE HUESO DENTAL (DOLARES)</t>
+  </si>
+  <si>
+    <t>MEMBRANA DE COLAGENO  (DOLARES)</t>
+  </si>
+  <si>
+    <t>PRF (PLASMA RICO EN FIBRINA)</t>
+  </si>
+  <si>
+    <t>CONSULTA POR ORTODONCIA</t>
+  </si>
+  <si>
+    <t>ORTODONCIA FIJA</t>
+  </si>
+  <si>
+    <t>ORTODONCIA FIJA LINGUAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORTODONCIA INTERCEPTIVA </t>
+  </si>
+  <si>
+    <t>PLACA CONTENCION PARA ORTOD. X PLACA</t>
+  </si>
+  <si>
+    <t>MINI IMPLANTE C/UNO</t>
+  </si>
+  <si>
+    <t>ORTODONCIA</t>
+  </si>
+  <si>
+    <t>REM.CUERP EXTR.(MUC. TEJI ALVEOLAR SUBCUT)</t>
+  </si>
+  <si>
+    <t>PATOLOGIAS</t>
+  </si>
+  <si>
+    <t>ODONTOLOGÍA - OTROS</t>
+  </si>
+  <si>
+    <t>CERT. DIAGNÓSTICO MÉD.</t>
+  </si>
+  <si>
+    <t>COPIA REP. OPERATORIO</t>
+  </si>
+  <si>
+    <t>530</t>
+  </si>
+  <si>
+    <t>EE. INLASER OSIRIS</t>
+  </si>
+  <si>
+    <t>REFRACTIVA</t>
+  </si>
+  <si>
+    <t>532</t>
+  </si>
+  <si>
+    <t>EE. INLASER OCT CEL GANGLIONARES</t>
+  </si>
+  <si>
+    <t>EXAMENES ESPECIALES</t>
+  </si>
+  <si>
+    <t>533</t>
+  </si>
+  <si>
+    <t>EE - ULTRABIOM (UBM)</t>
+  </si>
+  <si>
+    <t>609</t>
+  </si>
+  <si>
+    <t>EST. LENTES</t>
+  </si>
+  <si>
+    <t>OPTICA</t>
+  </si>
+  <si>
+    <t>195</t>
+  </si>
+  <si>
+    <t>EXAMEN ESP OFTALM OCT CELULAS GLANGLIONARES</t>
+  </si>
+  <si>
+    <t>OFTALMOLOGIA</t>
+  </si>
+  <si>
+    <t>DOCUMENTOS</t>
+  </si>
+  <si>
+    <t>427</t>
+  </si>
+  <si>
+    <t>F - P.E. OCP. TRIAMCINOLONA</t>
+  </si>
+  <si>
+    <t>OCULOPLASTIA</t>
+  </si>
+  <si>
+    <t>144</t>
+  </si>
+  <si>
+    <t>145</t>
+  </si>
+  <si>
+    <t>F - P.E. TAP. LAGRIMAL</t>
+  </si>
+  <si>
+    <t>F - P.E. TRIAMCINOLONA</t>
+  </si>
+  <si>
+    <t>173</t>
+  </si>
+  <si>
+    <t>F - QX - OFT. CROSS + PTK</t>
+  </si>
+  <si>
+    <t>135</t>
+  </si>
+  <si>
+    <t>F-EE-ULTRABIOM (UBM)</t>
+  </si>
+  <si>
+    <t>146</t>
+  </si>
+  <si>
+    <t>F. P.E. VABYSMO</t>
+  </si>
+  <si>
+    <t>262</t>
+  </si>
+  <si>
+    <t>265</t>
+  </si>
+  <si>
+    <t>266</t>
+  </si>
+  <si>
+    <t>Qx - GLAU RECUB. VALV.</t>
+  </si>
+  <si>
+    <t>GLAUCOMA</t>
+  </si>
+  <si>
+    <t>QX - GLAU EXTRAC. VALVULA</t>
+  </si>
+  <si>
+    <t>QX - GLAU NEEDLING</t>
   </si>
 </sst>
 </file>
@@ -7063,8 +7447,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7361,11 +7746,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1312"/>
+  <dimension ref="A1:D1419"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="33.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" style="1"/>
+    <col min="2" max="2" width="45.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -25736,7 +26122,1503 @@
         <v>97</v>
       </c>
     </row>
+    <row r="1313" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1313" s="1">
+        <v>800</v>
+      </c>
+      <c r="B1313" t="s">
+        <v>2336</v>
+      </c>
+      <c r="C1313" t="s">
+        <v>2338</v>
+      </c>
+      <c r="D1313" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1314" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1314" s="1">
+        <v>801</v>
+      </c>
+      <c r="B1314" t="s">
+        <v>2337</v>
+      </c>
+      <c r="C1314" t="s">
+        <v>2338</v>
+      </c>
+      <c r="D1314" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1315" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1315" s="1">
+        <v>805</v>
+      </c>
+      <c r="B1315" t="s">
+        <v>2339</v>
+      </c>
+      <c r="C1315" t="s">
+        <v>2343</v>
+      </c>
+      <c r="D1315" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1316" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1316" s="1">
+        <v>806</v>
+      </c>
+      <c r="B1316" t="s">
+        <v>2340</v>
+      </c>
+      <c r="C1316" t="s">
+        <v>2343</v>
+      </c>
+      <c r="D1316" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1317" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1317" s="1">
+        <v>807</v>
+      </c>
+      <c r="B1317" t="s">
+        <v>2341</v>
+      </c>
+      <c r="C1317" t="s">
+        <v>2343</v>
+      </c>
+      <c r="D1317" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1318" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1318" s="1">
+        <v>808</v>
+      </c>
+      <c r="B1318" t="s">
+        <v>1675</v>
+      </c>
+      <c r="C1318" t="s">
+        <v>2343</v>
+      </c>
+      <c r="D1318" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1319" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1319" s="1">
+        <v>809</v>
+      </c>
+      <c r="B1319" t="s">
+        <v>2342</v>
+      </c>
+      <c r="C1319" t="s">
+        <v>2343</v>
+      </c>
+      <c r="D1319" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1320" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1320" s="1">
+        <v>815</v>
+      </c>
+      <c r="B1320" t="s">
+        <v>2344</v>
+      </c>
+      <c r="C1320" t="s">
+        <v>2347</v>
+      </c>
+      <c r="D1320" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1321" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1321" s="1">
+        <v>816</v>
+      </c>
+      <c r="B1321" t="s">
+        <v>2345</v>
+      </c>
+      <c r="C1321" t="s">
+        <v>2347</v>
+      </c>
+      <c r="D1321" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1322" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1322" s="1">
+        <v>817</v>
+      </c>
+      <c r="B1322" t="s">
+        <v>2346</v>
+      </c>
+      <c r="C1322" t="s">
+        <v>2347</v>
+      </c>
+      <c r="D1322" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1323" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1323" s="1">
+        <v>820</v>
+      </c>
+      <c r="B1323" t="s">
+        <v>2348</v>
+      </c>
+      <c r="C1323" t="s">
+        <v>2354</v>
+      </c>
+      <c r="D1323" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1324" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1324" s="1">
+        <v>821</v>
+      </c>
+      <c r="B1324" t="s">
+        <v>2349</v>
+      </c>
+      <c r="C1324" t="s">
+        <v>2354</v>
+      </c>
+      <c r="D1324" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1325" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1325" s="1">
+        <v>822</v>
+      </c>
+      <c r="B1325" t="s">
+        <v>2350</v>
+      </c>
+      <c r="C1325" t="s">
+        <v>2354</v>
+      </c>
+      <c r="D1325" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1326" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1326" s="1">
+        <v>823</v>
+      </c>
+      <c r="B1326" t="s">
+        <v>2351</v>
+      </c>
+      <c r="C1326" t="s">
+        <v>2354</v>
+      </c>
+      <c r="D1326" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1327" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1327" s="1">
+        <v>824</v>
+      </c>
+      <c r="B1327" t="s">
+        <v>2352</v>
+      </c>
+      <c r="C1327" t="s">
+        <v>2354</v>
+      </c>
+      <c r="D1327" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1328" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1328" s="1">
+        <v>825</v>
+      </c>
+      <c r="B1328" t="s">
+        <v>2353</v>
+      </c>
+      <c r="C1328" t="s">
+        <v>2354</v>
+      </c>
+      <c r="D1328" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1329" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1329" s="1">
+        <v>830</v>
+      </c>
+      <c r="B1329" t="s">
+        <v>1669</v>
+      </c>
+      <c r="C1329" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1329" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1330" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1330" s="1">
+        <v>831</v>
+      </c>
+      <c r="B1330" t="s">
+        <v>2355</v>
+      </c>
+      <c r="C1330" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1330" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1331" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1331" s="1">
+        <v>832</v>
+      </c>
+      <c r="B1331" t="s">
+        <v>2356</v>
+      </c>
+      <c r="C1331" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1331" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1332" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1332" s="1">
+        <v>833</v>
+      </c>
+      <c r="B1332" t="s">
+        <v>2357</v>
+      </c>
+      <c r="C1332" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1332" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1333" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1333" s="1">
+        <v>834</v>
+      </c>
+      <c r="B1333" t="s">
+        <v>2358</v>
+      </c>
+      <c r="C1333" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1333" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1334" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1334" s="1">
+        <v>835</v>
+      </c>
+      <c r="B1334" t="s">
+        <v>2359</v>
+      </c>
+      <c r="C1334" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1334" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1335" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1335" s="1">
+        <v>836</v>
+      </c>
+      <c r="B1335" t="s">
+        <v>2360</v>
+      </c>
+      <c r="C1335" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1335" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1336" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1336" s="1">
+        <v>837</v>
+      </c>
+      <c r="B1336" t="s">
+        <v>2361</v>
+      </c>
+      <c r="C1336" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1336" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1337" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1337" s="1">
+        <v>838</v>
+      </c>
+      <c r="B1337" t="s">
+        <v>2362</v>
+      </c>
+      <c r="C1337" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1337" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1338" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1338" s="1">
+        <v>845</v>
+      </c>
+      <c r="B1338" t="s">
+        <v>2364</v>
+      </c>
+      <c r="C1338" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1338" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1339" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1339" s="1">
+        <v>846</v>
+      </c>
+      <c r="B1339" t="s">
+        <v>2365</v>
+      </c>
+      <c r="C1339" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1339" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1340" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1340" s="1">
+        <v>847</v>
+      </c>
+      <c r="B1340" t="s">
+        <v>2366</v>
+      </c>
+      <c r="C1340" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1340" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1341" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1341" s="1">
+        <v>848</v>
+      </c>
+      <c r="B1341" t="s">
+        <v>2367</v>
+      </c>
+      <c r="C1341" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1341" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1342" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1342" s="1">
+        <v>849</v>
+      </c>
+      <c r="B1342" t="s">
+        <v>2368</v>
+      </c>
+      <c r="C1342" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1342" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1343" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1343" s="1">
+        <v>850</v>
+      </c>
+      <c r="B1343" t="s">
+        <v>2369</v>
+      </c>
+      <c r="C1343" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1343" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1344" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1344" s="1">
+        <v>851</v>
+      </c>
+      <c r="B1344" t="s">
+        <v>2370</v>
+      </c>
+      <c r="C1344" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1344" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1345" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1345" s="1">
+        <v>852</v>
+      </c>
+      <c r="B1345" t="s">
+        <v>2371</v>
+      </c>
+      <c r="C1345" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1345" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1346" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1346" s="1">
+        <v>853</v>
+      </c>
+      <c r="B1346" t="s">
+        <v>2372</v>
+      </c>
+      <c r="C1346" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1346" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1347" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1347" s="1">
+        <v>854</v>
+      </c>
+      <c r="B1347" t="s">
+        <v>2373</v>
+      </c>
+      <c r="C1347" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1347" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1348" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1348" s="1">
+        <v>855</v>
+      </c>
+      <c r="B1348" t="s">
+        <v>2374</v>
+      </c>
+      <c r="C1348" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1348" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1349" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1349" s="1">
+        <v>856</v>
+      </c>
+      <c r="B1349" t="s">
+        <v>2375</v>
+      </c>
+      <c r="C1349" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D1349" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1350" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1350" s="1">
+        <v>860</v>
+      </c>
+      <c r="B1350" t="s">
+        <v>2376</v>
+      </c>
+      <c r="C1350" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1350" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1351" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1351" s="1">
+        <v>861</v>
+      </c>
+      <c r="B1351" t="s">
+        <v>2377</v>
+      </c>
+      <c r="C1351" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1351" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1352" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1352" s="1">
+        <v>862</v>
+      </c>
+      <c r="B1352" t="s">
+        <v>2378</v>
+      </c>
+      <c r="C1352" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1352" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1353" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1353" s="1">
+        <v>863</v>
+      </c>
+      <c r="B1353" t="s">
+        <v>2379</v>
+      </c>
+      <c r="C1353" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1353" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1354" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1354" s="1">
+        <v>864</v>
+      </c>
+      <c r="B1354" t="s">
+        <v>2380</v>
+      </c>
+      <c r="C1354" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1354" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1355" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1355" s="1">
+        <v>865</v>
+      </c>
+      <c r="B1355" t="s">
+        <v>2381</v>
+      </c>
+      <c r="C1355" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1355" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1356" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1356" s="1">
+        <v>866</v>
+      </c>
+      <c r="B1356" t="s">
+        <v>2382</v>
+      </c>
+      <c r="C1356" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1356" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1357" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1357" s="1">
+        <v>867</v>
+      </c>
+      <c r="B1357" t="s">
+        <v>2383</v>
+      </c>
+      <c r="C1357" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1357" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1358" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1358" s="1">
+        <v>868</v>
+      </c>
+      <c r="B1358" t="s">
+        <v>2384</v>
+      </c>
+      <c r="C1358" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1358" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1359" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1359" s="1">
+        <v>869</v>
+      </c>
+      <c r="B1359" t="s">
+        <v>2385</v>
+      </c>
+      <c r="C1359" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1359" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1360" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1360" s="1">
+        <v>870</v>
+      </c>
+      <c r="B1360" t="s">
+        <v>2386</v>
+      </c>
+      <c r="C1360" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1360" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1361" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1361" s="1">
+        <v>871</v>
+      </c>
+      <c r="B1361" t="s">
+        <v>2387</v>
+      </c>
+      <c r="C1361" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1361" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1362" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1362" s="1">
+        <v>872</v>
+      </c>
+      <c r="B1362" t="s">
+        <v>2388</v>
+      </c>
+      <c r="C1362" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1362" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1363" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1363" s="1">
+        <v>873</v>
+      </c>
+      <c r="B1363" t="s">
+        <v>2389</v>
+      </c>
+      <c r="C1363" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1363" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1364" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1364" s="1">
+        <v>874</v>
+      </c>
+      <c r="B1364" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C1364" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1364" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1365" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1365" s="1">
+        <v>875</v>
+      </c>
+      <c r="B1365" t="s">
+        <v>2391</v>
+      </c>
+      <c r="C1365" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1365" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1366" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1366" s="1">
+        <v>876</v>
+      </c>
+      <c r="B1366" t="s">
+        <v>2392</v>
+      </c>
+      <c r="C1366" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1366" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1367" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1367" s="1">
+        <v>880</v>
+      </c>
+      <c r="B1367" t="s">
+        <v>2394</v>
+      </c>
+      <c r="C1367" t="s">
+        <v>2402</v>
+      </c>
+      <c r="D1367" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1368" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1368" s="1">
+        <v>881</v>
+      </c>
+      <c r="B1368" t="s">
+        <v>2395</v>
+      </c>
+      <c r="C1368" t="s">
+        <v>2402</v>
+      </c>
+      <c r="D1368" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1369" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1369" s="1">
+        <v>882</v>
+      </c>
+      <c r="B1369" t="s">
+        <v>2396</v>
+      </c>
+      <c r="C1369" t="s">
+        <v>2402</v>
+      </c>
+      <c r="D1369" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1370" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1370" s="1">
+        <v>883</v>
+      </c>
+      <c r="B1370" t="s">
+        <v>2397</v>
+      </c>
+      <c r="C1370" t="s">
+        <v>2402</v>
+      </c>
+      <c r="D1370" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1371" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1371" s="1">
+        <v>884</v>
+      </c>
+      <c r="B1371" t="s">
+        <v>2398</v>
+      </c>
+      <c r="C1371" t="s">
+        <v>2402</v>
+      </c>
+      <c r="D1371" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1372" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1372" s="1">
+        <v>885</v>
+      </c>
+      <c r="B1372" t="s">
+        <v>2399</v>
+      </c>
+      <c r="C1372" t="s">
+        <v>2402</v>
+      </c>
+      <c r="D1372" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1373" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1373" s="1">
+        <v>886</v>
+      </c>
+      <c r="B1373" t="s">
+        <v>2400</v>
+      </c>
+      <c r="C1373" t="s">
+        <v>2402</v>
+      </c>
+      <c r="D1373" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1374" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1374" s="1">
+        <v>887</v>
+      </c>
+      <c r="B1374" t="s">
+        <v>2401</v>
+      </c>
+      <c r="C1374" t="s">
+        <v>2402</v>
+      </c>
+      <c r="D1374" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1375" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1375" s="1">
+        <v>890</v>
+      </c>
+      <c r="B1375" t="s">
+        <v>2403</v>
+      </c>
+      <c r="C1375" t="s">
+        <v>2409</v>
+      </c>
+      <c r="D1375" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1376" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1376" s="1">
+        <v>891</v>
+      </c>
+      <c r="B1376" t="s">
+        <v>2404</v>
+      </c>
+      <c r="C1376" t="s">
+        <v>2409</v>
+      </c>
+      <c r="D1376" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1377" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1377" s="1">
+        <v>892</v>
+      </c>
+      <c r="B1377" t="s">
+        <v>2405</v>
+      </c>
+      <c r="C1377" t="s">
+        <v>2409</v>
+      </c>
+      <c r="D1377" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1378" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1378" s="1">
+        <v>893</v>
+      </c>
+      <c r="B1378" t="s">
+        <v>2406</v>
+      </c>
+      <c r="C1378" t="s">
+        <v>2409</v>
+      </c>
+      <c r="D1378" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1379" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1379" s="1">
+        <v>894</v>
+      </c>
+      <c r="B1379" t="s">
+        <v>2407</v>
+      </c>
+      <c r="C1379" t="s">
+        <v>2409</v>
+      </c>
+      <c r="D1379" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1380" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1380" s="1">
+        <v>895</v>
+      </c>
+      <c r="B1380" t="s">
+        <v>2408</v>
+      </c>
+      <c r="C1380" t="s">
+        <v>2409</v>
+      </c>
+      <c r="D1380" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1381" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1381" s="1">
+        <v>896</v>
+      </c>
+      <c r="B1381" t="s">
+        <v>2410</v>
+      </c>
+      <c r="C1381" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1381" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1382" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1382" s="1">
+        <v>897</v>
+      </c>
+      <c r="B1382" t="s">
+        <v>2411</v>
+      </c>
+      <c r="C1382" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1382" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1383" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1383" s="1">
+        <v>898</v>
+      </c>
+      <c r="B1383" t="s">
+        <v>2412</v>
+      </c>
+      <c r="C1383" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1383" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1384" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1384" s="1">
+        <v>899</v>
+      </c>
+      <c r="B1384" t="s">
+        <v>2413</v>
+      </c>
+      <c r="C1384" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1384" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1385" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1385" s="1">
+        <v>900</v>
+      </c>
+      <c r="B1385" t="s">
+        <v>2414</v>
+      </c>
+      <c r="C1385" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1385" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1386" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1386" s="1">
+        <v>901</v>
+      </c>
+      <c r="B1386" t="s">
+        <v>2415</v>
+      </c>
+      <c r="C1386" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1386" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1387" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1387" s="1">
+        <v>910</v>
+      </c>
+      <c r="B1387" t="s">
+        <v>2416</v>
+      </c>
+      <c r="C1387" t="s">
+        <v>2422</v>
+      </c>
+      <c r="D1387" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1388" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1388" s="1">
+        <v>911</v>
+      </c>
+      <c r="B1388" t="s">
+        <v>2417</v>
+      </c>
+      <c r="C1388" t="s">
+        <v>2422</v>
+      </c>
+      <c r="D1388" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1389" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1389" s="1">
+        <v>912</v>
+      </c>
+      <c r="B1389" t="s">
+        <v>2418</v>
+      </c>
+      <c r="C1389" t="s">
+        <v>2422</v>
+      </c>
+      <c r="D1389" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1390" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1390" s="1">
+        <v>913</v>
+      </c>
+      <c r="B1390" t="s">
+        <v>2419</v>
+      </c>
+      <c r="C1390" t="s">
+        <v>2422</v>
+      </c>
+      <c r="D1390" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1391" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1391" s="1">
+        <v>914</v>
+      </c>
+      <c r="B1391" t="s">
+        <v>2420</v>
+      </c>
+      <c r="C1391" t="s">
+        <v>2422</v>
+      </c>
+      <c r="D1391" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1392" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1392" s="1">
+        <v>915</v>
+      </c>
+      <c r="B1392" t="s">
+        <v>2421</v>
+      </c>
+      <c r="C1392" t="s">
+        <v>2422</v>
+      </c>
+      <c r="D1392" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1393" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1393" s="1">
+        <v>920</v>
+      </c>
+      <c r="B1393" t="s">
+        <v>2423</v>
+      </c>
+      <c r="C1393" t="s">
+        <v>2424</v>
+      </c>
+      <c r="D1393" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1394" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1394" s="1">
+        <v>930</v>
+      </c>
+      <c r="B1394" t="s">
+        <v>2425</v>
+      </c>
+      <c r="C1394" t="s">
+        <v>1671</v>
+      </c>
+      <c r="D1394" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1395" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1395" s="1">
+        <v>935</v>
+      </c>
+      <c r="B1395" t="s">
+        <v>1914</v>
+      </c>
+      <c r="C1395" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1395" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1396" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1396" s="1">
+        <v>936</v>
+      </c>
+      <c r="B1396" t="s">
+        <v>2426</v>
+      </c>
+      <c r="C1396" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1396" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1397" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1397" s="1">
+        <v>937</v>
+      </c>
+      <c r="B1397" t="s">
+        <v>1918</v>
+      </c>
+      <c r="C1397" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1397" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1398" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1398" s="1">
+        <v>938</v>
+      </c>
+      <c r="B1398" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1398" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1398" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1399" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1399" s="1">
+        <v>939</v>
+      </c>
+      <c r="B1399" t="s">
+        <v>1920</v>
+      </c>
+      <c r="C1399" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1399" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1400" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1400" s="1">
+        <v>940</v>
+      </c>
+      <c r="B1400" t="s">
+        <v>1922</v>
+      </c>
+      <c r="C1400" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1400" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1401" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1401" s="1">
+        <v>941</v>
+      </c>
+      <c r="B1401" t="s">
+        <v>1924</v>
+      </c>
+      <c r="C1401" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1401" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1402" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1402" s="1">
+        <v>942</v>
+      </c>
+      <c r="B1402" t="s">
+        <v>1926</v>
+      </c>
+      <c r="C1402" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1402" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1403" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1403" s="1">
+        <v>943</v>
+      </c>
+      <c r="B1403" t="s">
+        <v>1928</v>
+      </c>
+      <c r="C1403" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1403" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1404" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1404" s="1">
+        <v>944</v>
+      </c>
+      <c r="B1404" t="s">
+        <v>2427</v>
+      </c>
+      <c r="C1404" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1404" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1405" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1405" s="1">
+        <v>945</v>
+      </c>
+      <c r="B1405" t="s">
+        <v>1930</v>
+      </c>
+      <c r="C1405" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1405" t="s">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="1406" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1406" s="1" t="s">
+        <v>2428</v>
+      </c>
+      <c r="B1406" t="s">
+        <v>2429</v>
+      </c>
+      <c r="C1406" t="s">
+        <v>2433</v>
+      </c>
+      <c r="D1406" t="s">
+        <v>2430</v>
+      </c>
+    </row>
+    <row r="1407" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1407" s="1" t="s">
+        <v>2431</v>
+      </c>
+      <c r="B1407" t="s">
+        <v>2432</v>
+      </c>
+      <c r="C1407" t="s">
+        <v>2433</v>
+      </c>
+      <c r="D1407" t="s">
+        <v>2430</v>
+      </c>
+    </row>
+    <row r="1408" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1408" s="1" t="s">
+        <v>2434</v>
+      </c>
+      <c r="B1408" t="s">
+        <v>2435</v>
+      </c>
+      <c r="C1408" t="s">
+        <v>2433</v>
+      </c>
+      <c r="D1408" t="s">
+        <v>2430</v>
+      </c>
+    </row>
+    <row r="1409" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1409" s="1" t="s">
+        <v>2436</v>
+      </c>
+      <c r="B1409" t="s">
+        <v>2437</v>
+      </c>
+      <c r="D1409" t="s">
+        <v>2438</v>
+      </c>
+    </row>
+    <row r="1410" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1410" s="1" t="s">
+        <v>2439</v>
+      </c>
+      <c r="B1410" t="s">
+        <v>2440</v>
+      </c>
+      <c r="C1410" t="s">
+        <v>2442</v>
+      </c>
+      <c r="D1410" t="s">
+        <v>2441</v>
+      </c>
+    </row>
+    <row r="1411" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1411" s="1" t="s">
+        <v>2443</v>
+      </c>
+      <c r="B1411" t="s">
+        <v>2444</v>
+      </c>
+      <c r="C1411" t="s">
+        <v>2338</v>
+      </c>
+      <c r="D1411" t="s">
+        <v>2445</v>
+      </c>
+    </row>
+    <row r="1412" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1412" s="1" t="s">
+        <v>2446</v>
+      </c>
+      <c r="B1412" t="s">
+        <v>2448</v>
+      </c>
+      <c r="C1412" t="s">
+        <v>2338</v>
+      </c>
+      <c r="D1412" t="s">
+        <v>2441</v>
+      </c>
+    </row>
+    <row r="1413" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1413" s="1" t="s">
+        <v>2447</v>
+      </c>
+      <c r="B1413" t="s">
+        <v>2449</v>
+      </c>
+      <c r="C1413" t="s">
+        <v>2338</v>
+      </c>
+      <c r="D1413" t="s">
+        <v>2441</v>
+      </c>
+    </row>
+    <row r="1414" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1414" s="1" t="s">
+        <v>2450</v>
+      </c>
+      <c r="B1414" t="s">
+        <v>2451</v>
+      </c>
+      <c r="C1414" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1414" t="s">
+        <v>2441</v>
+      </c>
+    </row>
+    <row r="1415" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1415" s="1" t="s">
+        <v>2452</v>
+      </c>
+      <c r="B1415" t="s">
+        <v>2453</v>
+      </c>
+      <c r="C1415" t="s">
+        <v>2433</v>
+      </c>
+      <c r="D1415" t="s">
+        <v>2441</v>
+      </c>
+    </row>
+    <row r="1416" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1416" s="1" t="s">
+        <v>2454</v>
+      </c>
+      <c r="B1416" t="s">
+        <v>2455</v>
+      </c>
+      <c r="C1416" t="s">
+        <v>2338</v>
+      </c>
+      <c r="D1416" t="s">
+        <v>2441</v>
+      </c>
+    </row>
+    <row r="1417" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1417" s="1" t="s">
+        <v>2456</v>
+      </c>
+      <c r="B1417" t="s">
+        <v>2459</v>
+      </c>
+      <c r="C1417" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1417" t="s">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="1418" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1418" s="1" t="s">
+        <v>2457</v>
+      </c>
+      <c r="B1418" t="s">
+        <v>2461</v>
+      </c>
+      <c r="C1418" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1418" t="s">
+        <v>2460</v>
+      </c>
+    </row>
+    <row r="1419" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1419" s="1" t="s">
+        <v>2458</v>
+      </c>
+      <c r="B1419" t="s">
+        <v>2462</v>
+      </c>
+      <c r="C1419" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1419" t="s">
+        <v>2460</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:D1405" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>